<commit_message>
feat(productos): Kit Plan Financiero v2.0 LIVE — 10 xlsx regenerados desde v1.1 (56 hojas, 2.437 fórmulas ×1,8, 9 gráficos, 25 rangos de CF, 60 validaciones, 56/56 hojas protegidas sin contraseña): tesorería encadenada + IVA trimestral calculado, informe bancario que calcula (P&L, cuadro francés con carencia, TIR/VAN/payback del proyecto, DSCR antes de deuda), resúmenes por referencia, semáforos honestos (ISNUMBER, «sin dato» ≠ 0), ratios con una sola tabla de umbrales. Gate offline 10/0, censo 0 defectos, decisión 14 en SPEC
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kK9BRAxpAsfsxudgwH42U
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-plan-financiero/02-calculadora-punto-equilibrio.xlsx
+++ b/astro-site/public/dl/kit-plan-financiero/02-calculadora-punto-equilibrio.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +95,31 @@
       <color rgb="001565C0"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -133,6 +156,21 @@
         <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D2D2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -160,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -225,10 +263,99 @@
     <xf numFmtId="165" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -299,6 +426,201 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Ingresos vs costes totales por cubiertos/día</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Break-Even'!B20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Break-Even'!$A$21:$A$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Break-Even'!$B$21:$B$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Break-Even'!C20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Break-Even'!$A$21:$A$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Break-Even'!$C$21:$C$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Break-Even'!D20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Break-Even'!$A$21:$A$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Break-Even'!$D$21:$D$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>€</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -591,11 +913,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="85" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -625,14 +947,14 @@
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>▸ En la pestaña 'Datos', introduce tus costes fijos mensuales, % de coste variable y ticket medio.</t>
+          <t>▸ En 'Datos' están los costes fijos OPERATIVOS. La cuota del préstamo va aparte (fila 15): el EBITDA se mide antes del servicio de deuda.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>▸ La pestaña 'Break-Even' calcula automáticamente la facturación mínima y cubiertos/día necesarios.</t>
+          <t>▸ 'Break-Even' da dos umbrales: el operativo (EBITDA = 0) y el de caja (con la cuota dentro), además del ticket medio necesario para tus cubiertos previstos.</t>
         </is>
       </c>
     </row>
@@ -654,7 +976,7 @@
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>▸ Costes Fijos: alquiler, nóminas fijas, seguros, cuotas — no varían con la actividad.</t>
+          <t>▸ Costes fijos: alquiler, personal fijo, seguros, gestoría — no varían con la actividad. La cuota del préstamo NO entra: es financiación, no explotación.</t>
         </is>
       </c>
     </row>
@@ -674,13 +996,35 @@
     </row>
     <row r="15"/>
     <row r="16">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-plan-financiero · info@aichef.pro</t>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>Todas las cifras van SIN IVA; en el 03 (tesorería) van CON IVA porque es caja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>Para editar una celda que no esté en verde: Revisar → Desproteger hoja (no tiene contraseña).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-plan-financiero · info@aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -705,9 +1049,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -724,7 +1068,13 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3">
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>VALORES DE EJEMPLO — sustitúyelos por los tuyos</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr"/>
       <c r="B4" s="6" t="inlineStr">
@@ -756,7 +1106,7 @@
           <t>Alquiler mensual</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="30" t="n">
         <v>3000</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -768,15 +1118,15 @@
     <row r="7">
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Nóminas fijas (bruto)</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n">
-        <v>12000</v>
+          <t>Coste total de personal fijo (salario bruto + SS empresa)</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="n">
+        <v>8800</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>€/mes — incluye SS empresa</t>
+          <t>€/mes — ≈ bruto × 1,32; es coste de EMPRESA, no bruto</t>
         </is>
       </c>
     </row>
@@ -786,7 +1136,7 @@
           <t>Seguros</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="30" t="n">
         <v>400</v>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -801,7 +1151,7 @@
           <t>Suministros (luz, agua, gas)</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="30" t="n">
         <v>1500</v>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -816,7 +1166,7 @@
           <t>Marketing fijo</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="30" t="n">
         <v>500</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -831,7 +1181,7 @@
           <t>Gestoría / Administración</t>
         </is>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="30" t="n">
         <v>300</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -841,19 +1191,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Cuota préstamo</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>800</v>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>€/mes</t>
-        </is>
-      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>La cuota del préstamo NO es un coste fijo operativo: va en la fila 15, fuera del EBITDA.</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="n"/>
+      <c r="D12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
@@ -861,7 +1205,7 @@
           <t>Otros gastos fijos</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="30" t="n">
         <v>500</v>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -873,17 +1217,31 @@
     <row r="14">
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>TOTAL COSTES FIJOS</t>
+          <t>TOTAL COSTES FIJOS OPERATIVOS</t>
         </is>
       </c>
       <c r="C14" s="12">
-        <f>SUM(C6:C13)</f>
-        <v>19000.0</v>
-      </c>
-    </row>
-    <row r="15"/>
+        <f>SUM(C6:C11)+C13</f>
+        <v>15000.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Cuota de préstamo (servicio de deuda)</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>800</v>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Cópiala del cuadro de amortización: 07!Financiación</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>COSTES VARIABLES</t>
         </is>
@@ -892,33 +1250,33 @@
     <row r="17">
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>% Coste Variable sobre ventas</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
+          <t>% Coste variable sobre ventas</t>
+        </is>
+      </c>
+      <c r="C17" s="34" t="n">
         <v>0.35</v>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Food cost + variable costs (30-40% típico)</t>
+          <t>Food cost + comisiones de delivery + variables (30-40 % típico). NO incluye el personal fijo.</t>
         </is>
       </c>
     </row>
     <row r="18"/>
     <row r="19">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>TICKET MEDIO</t>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>TICKET MEDIO (sin IVA)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Ticket medio por comensal</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="n">
+          <t>Ticket medio por comensal (€, sin IVA)</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="n">
         <v>22</v>
       </c>
     </row>
@@ -928,24 +1286,33 @@
           <t>Días de apertura al mes</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="C21" s="35" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="22"/>
     <row r="23"/>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="36" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A24:D24"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="1">
     <mergeCell ref="B1:D1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C6 C7 C8 C9 C10 C11 C13 C15 C20 C21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Importe no válido" error="Escribe un número mayor o igual que 0." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="C17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Porcentaje no válido" error="Escribe un porcentaje entre 0 y 1 (0,35 = 35 %)." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -966,11 +1333,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1005,67 +1372,67 @@
     <row r="5">
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Total Costes Fijos / mes</t>
+          <t>Total costes fijos operativos / mes</t>
         </is>
       </c>
       <c r="C5" s="15">
-        <f>Datos!C14</f>
-        <v>19000.0</v>
+        <f>Datos!$C$14</f>
+        <v>15000.0</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>% Coste Variable</t>
+          <t>% Coste variable</t>
         </is>
       </c>
       <c r="C6" s="16">
-        <f>Datos!C17</f>
+        <f>Datos!$C$17</f>
         <v>0.35</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Margen de Contribución</t>
+          <t>Margen de contribución</t>
         </is>
       </c>
       <c r="C7" s="16">
-        <f>1-Datos!C17</f>
+        <f>1-Datos!$C$17</f>
         <v>0.65</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>FACTURACIÓN BREAK-EVEN / mes</t>
+          <t>FACTURACIÓN BREAK-EVEN / mes (sin IVA)</t>
         </is>
       </c>
       <c r="C8" s="17">
-        <f>Datos!C14/(1-Datos!C17)</f>
-        <v>29230.76923076923</v>
+        <f>IFERROR(Datos!$C$14/(1-Datos!$C$17),"Revisa el % de coste variable (no puede ser 100 %)")</f>
+        <v>23076.923076923074</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Facturación Break-Even / día</t>
+          <t>Facturación break-even / día (sin IVA)</t>
         </is>
       </c>
       <c r="C9" s="15">
-        <f>C8/Datos!C21</f>
-        <v>1124.2603550295858</v>
+        <f>IFERROR($C$8/Datos!$C$21,"Indica los días de apertura")</f>
+        <v>887.5739644970413</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Cubiertos / día necesarios</t>
         </is>
       </c>
-      <c r="C10" s="18">
-        <f>C9/Datos!C20</f>
-        <v>51.102743410435714</v>
+      <c r="C10" s="37">
+        <f>IFERROR(ROUNDUP($C$9/Datos!$C$20,0),"Indica el ticket medio")</f>
+        <v>41.0</v>
       </c>
     </row>
     <row r="11">
@@ -1075,25 +1442,290 @@
         </is>
       </c>
       <c r="C11" s="18">
-        <f>C10*Datos!C21</f>
-        <v>1328.6713286713286</v>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
+        <f>IFERROR(ROUNDUP($C$8/Datos!$C$20,0),"—")</f>
+        <v>1049.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Cubiertos / día previstos</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Ticket medio necesario (€, sin IVA)</t>
+        </is>
+      </c>
+      <c r="C13" s="15">
+        <f>IFERROR($C$9/$C$12,"Indica los cubiertos/día previstos")</f>
+        <v>16.13770844540075</v>
+      </c>
+    </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>BREAK-EVEN DE CAJA (incluye la cuota del préstamo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Facturación break-even de caja / mes (sin IVA)</t>
+        </is>
+      </c>
+      <c r="C16" s="17">
+        <f>IFERROR((Datos!$C$14+Datos!$C$15)/(1-Datos!$C$17),"Revisa el % de coste variable (no puede ser 100 %)")</f>
+        <v>24307.69230769231</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Cubiertos / día para el break-even de caja</t>
+        </is>
+      </c>
+      <c r="C17" s="18">
+        <f>IFERROR(ROUNDUP($C$16/Datos!$C$21/Datos!$C$20,0),"Indica el ticket medio")</f>
+        <v>43.0</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>BLOQUE AUXILIAR DEL GRÁFICO — no lo edites</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>Cubiertos / día</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>Costes totales</t>
+        </is>
+      </c>
+      <c r="D20" s="40" t="inlineStr">
+        <is>
+          <t>Facturación break-even</t>
+        </is>
+      </c>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="41" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="42">
+        <f>IFERROR(ROUND($C$10*$F21,0),0)</f>
+        <v>10.0</v>
+      </c>
+      <c r="B21" s="43">
+        <f>IFERROR($A21*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>5720.0</v>
+      </c>
+      <c r="C21" s="43">
+        <f>IFERROR(Datos!$C$14+$B21*Datos!$C$17,0)</f>
+        <v>17002.0</v>
+      </c>
+      <c r="D21" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="44" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="42">
+        <f>IFERROR(ROUND($C$10*$F22,0),0)</f>
+        <v>21.0</v>
+      </c>
+      <c r="B22" s="43">
+        <f>IFERROR($A22*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>12012.0</v>
+      </c>
+      <c r="C22" s="43">
+        <f>IFERROR(Datos!$C$14+$B22*Datos!$C$17,0)</f>
+        <v>19204.2</v>
+      </c>
+      <c r="D22" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="44" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="42">
+        <f>IFERROR(ROUND($C$10*$F23,0),0)</f>
+        <v>31.0</v>
+      </c>
+      <c r="B23" s="43">
+        <f>IFERROR($A23*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>17732.0</v>
+      </c>
+      <c r="C23" s="43">
+        <f>IFERROR(Datos!$C$14+$B23*Datos!$C$17,0)</f>
+        <v>21206.2</v>
+      </c>
+      <c r="D23" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="44" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42">
+        <f>IFERROR(ROUND($C$10*$F24,0),0)</f>
+        <v>41.0</v>
+      </c>
+      <c r="B24" s="43">
+        <f>IFERROR($A24*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>23452.0</v>
+      </c>
+      <c r="C24" s="43">
+        <f>IFERROR(Datos!$C$14+$B24*Datos!$C$17,0)</f>
+        <v>23208.199999999997</v>
+      </c>
+      <c r="D24" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="42">
+        <f>IFERROR(ROUND($C$10*$F25,0),0)</f>
+        <v>51.0</v>
+      </c>
+      <c r="B25" s="43">
+        <f>IFERROR($A25*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>29172.0</v>
+      </c>
+      <c r="C25" s="43">
+        <f>IFERROR(Datos!$C$14+$B25*Datos!$C$17,0)</f>
+        <v>25210.199999999997</v>
+      </c>
+      <c r="D25" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E25" s="41" t="n"/>
+      <c r="F25" s="44" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="42">
+        <f>IFERROR(ROUND($C$10*$F26,0),0)</f>
+        <v>62.0</v>
+      </c>
+      <c r="B26" s="43">
+        <f>IFERROR($A26*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>35464.0</v>
+      </c>
+      <c r="C26" s="43">
+        <f>IFERROR(Datos!$C$14+$B26*Datos!$C$17,0)</f>
+        <v>27412.4</v>
+      </c>
+      <c r="D26" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="44" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42">
+        <f>IFERROR(ROUND($C$10*$F27,0),0)</f>
+        <v>72.0</v>
+      </c>
+      <c r="B27" s="43">
+        <f>IFERROR($A27*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>41184.0</v>
+      </c>
+      <c r="C27" s="43">
+        <f>IFERROR(Datos!$C$14+$B27*Datos!$C$17,0)</f>
+        <v>29414.4</v>
+      </c>
+      <c r="D27" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="44" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42">
+        <f>IFERROR(ROUND($C$10*$F28,0),0)</f>
+        <v>82.0</v>
+      </c>
+      <c r="B28" s="43">
+        <f>IFERROR($A28*Datos!$C$20*Datos!$C$21,0)</f>
+        <v>46904.0</v>
+      </c>
+      <c r="C28" s="43">
+        <f>IFERROR(Datos!$C$14+$B28*Datos!$C$17,0)</f>
+        <v>31416.399999999998</v>
+      </c>
+      <c r="D28" s="43">
+        <f>$C$8</f>
+        <v>23076.923076923074</v>
+      </c>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="44" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32"/>
   </sheetData>
-  <mergeCells count="2">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="1">
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="A15:C15"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Importe no válido" error="Escribe un número mayor o igual que 0." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -1104,6 +1736,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1114,11 +1747,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -1158,16 +1791,16 @@
     <row r="4">
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Ticket medio (€)</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="n">
+          <t>Ticket medio (€, sin IVA)</t>
+        </is>
+      </c>
+      <c r="C4" s="45" t="n">
         <v>18</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="46" t="n">
         <v>22</v>
       </c>
-      <c r="E4" s="21" t="n">
+      <c r="E4" s="47" t="n">
         <v>28</v>
       </c>
     </row>
@@ -1177,46 +1810,49 @@
           <t>Cubiertos / día</t>
         </is>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="48" t="n">
         <v>40</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="49" t="n">
         <v>55</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="50" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>% Coste Variable</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="n">
+          <t>% Coste variable (food + comisiones; NO incluye personal fijo)</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="n">
         <v>0.4</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="52" t="n">
         <v>0.35</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="53" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Costes Fijos / mes (€)</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="n">
-        <v>19000</v>
-      </c>
-      <c r="D7" s="20" t="n">
-        <v>19000</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>19000</v>
+          <t>Costes fijos operativos / mes (€) — de Datos!C14</t>
+        </is>
+      </c>
+      <c r="C7" s="19">
+        <f>Datos!$C$14</f>
+        <v>15000.0</v>
+      </c>
+      <c r="D7" s="20">
+        <f>Datos!$C$14</f>
+        <v>15000.0</v>
+      </c>
+      <c r="E7" s="21">
+        <f>Datos!$C$14</f>
+        <v>15000.0</v>
       </c>
     </row>
     <row r="8"/>
@@ -1230,19 +1866,19 @@
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Facturación mensual</t>
+          <t>Facturación mensual (sin IVA)</t>
         </is>
       </c>
       <c r="C10" s="17">
-        <f>C4*C5*26</f>
+        <f>C4*C5*Datos!$C$21</f>
         <v>18720.0</v>
       </c>
       <c r="D10" s="17">
-        <f>D4*D5*26</f>
+        <f>D4*D5*Datos!$C$21</f>
         <v>31460.0</v>
       </c>
       <c r="E10" s="17">
-        <f>E4*E5*26</f>
+        <f>E4*E5*Datos!$C$21</f>
         <v>54600.0</v>
       </c>
     </row>
@@ -1292,31 +1928,103 @@
       </c>
       <c r="C13" s="12">
         <f>C12-C7</f>
-        <v>-7768.0</v>
+        <v>-3768.0</v>
       </c>
       <c r="D13" s="12">
         <f>D12-D7</f>
-        <v>1449.0</v>
+        <v>5449.0</v>
       </c>
       <c r="E13" s="12">
         <f>E12-E7</f>
-        <v>19220.0</v>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15"/>
+        <v>23220.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cuota de préstamo (servicio de deuda)</t>
+        </is>
+      </c>
+      <c r="C14" s="54">
+        <f>Datos!$C$15</f>
+        <v>800.0</v>
+      </c>
+      <c r="D14" s="54">
+        <f>Datos!$C$15</f>
+        <v>800.0</v>
+      </c>
+      <c r="E14" s="54">
+        <f>Datos!$C$15</f>
+        <v>800.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>RESULTADO DESPUÉS DE DEUDA</t>
+        </is>
+      </c>
+      <c r="C15" s="54">
+        <f>C13-C14</f>
+        <v>-4568.0</v>
+      </c>
+      <c r="D15" s="54">
+        <f>D13-D14</f>
+        <v>4649.0</v>
+      </c>
+      <c r="E15" s="54">
+        <f>E13-E14</f>
+        <v>22420.0</v>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Margen EBITDA %</t>
+        </is>
+      </c>
+      <c r="C16" s="55">
+        <f>IF(C10=0,"",C13/C10)</f>
+        <v>-0.2012820512820513</v>
+      </c>
+      <c r="D16" s="55">
+        <f>IF(D10=0,"",D13/D10)</f>
+        <v>0.17320406865861412</v>
+      </c>
+      <c r="E16" s="55">
+        <f>IF(E10=0,"",E13/E10)</f>
+        <v>0.42527472527472526</v>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="B18" s="56" t="inlineStr">
+        <is>
+          <t>El EBITDA de la fila 13 va ANTES del servicio de deuda: es el que se compara con los benchmarks del 06 y del 07.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="36" t="inlineStr">
         <is>
           <t>© 2026 AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A16:E16"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <mergeCells count="1">
     <mergeCell ref="B1:E1"/>
   </mergeCells>
+  <conditionalFormatting sqref="C13:E13">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>=C13&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>